<commit_message>
fix: restore missing anime metadata and refine description panel layout
</commit_message>
<xml_diff>
--- a/assets/data/anime.xlsx
+++ b/assets/data/anime.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q107"/>
+  <dimension ref="A1:R107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -502,6 +502,11 @@
           <t>Fav</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -575,6 +580,11 @@
       <c r="Q2" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Two teenagers share a profound, magical connection upon discovering they are swapping bodies.</t>
         </is>
       </c>
     </row>
@@ -652,6 +662,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>A young girl teams up with a mysterious young man to close magical doors causing disasters across Japan.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -727,6 +742,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>An aloof boy discovers his popular classmate is secretly suffering from a fatal pancreatic illness.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -802,6 +822,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>A runaway high school boy in Tokyo meets a girl who has the power to manipulate the weather.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -877,6 +902,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>A student aspiring to be a shoemaker and a mysterious older woman find solace in each other on rainy mornings.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -952,6 +982,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Two seemingly very different high schoolers discover each other's hidden sides and form a close bond.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1027,6 +1062,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>A kind-hearted boy becomes a demon slayer to avenge his family and cure his demon-turned sister.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1102,6 +1142,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>A piano prodigy who lost his ability to hear the piano meets a free-spirited violinist who brings color back to his life.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1177,6 +1222,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Two teenagers investigate a mysterious tunnel that can grant wishes, but at a heavy cost of time.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1252,6 +1302,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>A surfer and a firefighter fall in love, but tragedy strikes, leading to supernatural encounters.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1327,6 +1382,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>A poignant tale of two childhood friends drifting apart over time and distance.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1402,6 +1462,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>A high schooler helps girls suffering from "Puberty Syndrome," starting with a forgotten teen actress.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1477,6 +1542,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>A doll-artisan enthusiast helps his popular classmate create cosplay outfits, blossoming into a sweet romance.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1552,6 +1622,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>A young girl befriends a forest spirit who will disappear forever if touched by a human.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1627,6 +1702,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Two eccentric high schoolers get entangled in insane battles involving ghosts and aliens.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1702,6 +1782,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>A beautifully animated reimagining of the classic Japanese folktale of the Bamboo Cutter.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1777,6 +1862,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>A sci-fi romance exploring parallel universes and the choices that define true love.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1852,6 +1942,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>The companion piece to "To Every You", showing the alternate universe path of love and sacrifice.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1927,6 +2022,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>A street kid survives in a technology-obsessed city of the future by becoming a mercenary outlaw.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2002,6 +2102,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Set in the League of Legends universe, two sisters fight on rival sides of a war between two cities.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2077,6 +2182,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>A former bully seeks redemption by trying to befriend the deaf girl he tormented in elementary school.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2147,6 +2257,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>A heartbreaking story of two siblings struggling to survive in Japan during the final months of WWII.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2217,6 +2332,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>A girl who lost her voice magically after traumatizing her family learns to express herself through music.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2287,6 +2407,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Humanity fights for survival against terrifying giant humanoids known as Titans.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2357,6 +2482,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Childhood friends from a sea village must attend school on the surface, causing friction and romance.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2427,6 +2557,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>An energy-conserving high schooler joins the classic literature club and solves everyday mysteries.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2497,6 +2632,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>In a post-apocalyptic future, children pilot giant mechs to defend humanity against monstrous threats.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2567,6 +2707,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>A young man is transported to a fantasy world with the ability to rewind time upon his death.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2637,6 +2782,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>A group of friends explore the nature of fireworks while a boy uses a mysterious orb to alter time.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2707,6 +2857,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>A high schooler travels back in time to help his past self correct a mistake and save his love.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2777,6 +2932,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Three troubled teens seek out an urban legend known as the Summer Ghost to find answers about life and death.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2847,6 +3007,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>A beautiful, emotional one-shot about the complicated rivalry and friendship of two aspiring manga artists.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2917,6 +3082,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>A young viking warrior seeks revenge against the man who killed his father in a deeply philosophical historical epic.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2987,6 +3157,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>A brilliant high school student discovers a supernatural notebook that kills anyone whose name is written in it.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3057,6 +3232,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>A delinquent student finds meaning in life by helping a sweet, chronically ill girl revive the school drama club.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -3127,6 +3307,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Two students suffering from insomnia find comfort in each other and the school's abandoned observatory.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -3197,6 +3382,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>A sharp-witted apothecary girl solves medical mysteries and political intrigue within the Emperor's inner palace.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -3267,6 +3457,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>A high schooler consumes a cursed talisman and gets drawn into a dangerous world of Curses and Sorcerers.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -3337,6 +3532,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Childhood friends reconnect years later to help the spirit of their deceased friend pass on.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -3407,6 +3607,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Two awkward coworkers fake an engagement to avoid being transferred to a branch office in Siberia.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3477,6 +3682,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>A sweet sports romance about a badminton player and a basketball star living under the same roof.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3547,6 +3757,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>An apathetic high school boy is slowly won over by his perfect, angelic neighbor who starts cooking for him.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -3617,6 +3832,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>A socially awkward boy with dark fantasies slowly falls in love with the quirky, popular girl in his class.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3687,6 +3907,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Two mismatched students are paired up for a bizarre "marriage practical" assignment in school.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3757,6 +3982,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Two brilliant student council leaders try to trick each other into confessing their love first.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -3827,6 +4057,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Two mismatched high schoolers team up to help each other confess to their respective crushes.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3897,6 +4132,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>A man travels back in time to his childhood to solve a string of kidnappings and save his classmate.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3967,6 +4207,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Students in an ultra-competitive, cutthroat high school must use deception and strategy to rise to the top.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -4037,6 +4282,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>A spy, an assassin, and a telepathic child pretend to be a normal family for a high-stakes mission.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -4107,6 +4357,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>A beautiful half-Russian girl mutters sweet things in Russian, unaware that her crush perfectly understands her.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -4177,6 +4432,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>A heartwarming romance between a student at a boys' delinquent school and a girl from an elite academy.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -4247,6 +4507,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>A young woman cursed with an old body gets swept up in the magical world of a wizard named Howl.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -4317,6 +4582,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>A young man merges with his pet chainsaw devil and joins a government agency to hunt other devils.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -4387,6 +4657,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>A boy constantly finds himself comforting the girls who lose the "love triangles" in his school.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -4457,6 +4732,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>A marine biology student becomes the caretaker for a stubborn, wheelchair-bound artist with big dreams.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -4527,6 +4807,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>A happy alien tries to bring joy to a deeply traumatized human girl, leading to a dark tragedy.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -4597,6 +4882,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>A touching drama about connection and finding light in a dark world.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -4667,6 +4957,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>A comedic misunderstanding between two friends leads to unexpected romance.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -4737,6 +5032,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>An emotional drama focused on terminal illness, love, and living life to the fullest.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -4807,6 +5107,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Childhood friends must navigate their shifting feelings and break the cycle of a complicated game.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -4877,6 +5182,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>A secret organization of highly trained schoolgirls works in the shadows to maintain peace in Japan.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -4947,6 +5257,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>A fierce delinquent joins a high school famous for brawling to fight for the town's safety.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -5017,6 +5332,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>A soul is given a second chance at life inhabiting the body of a suicidal middle schooler.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -5087,6 +5407,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Child soldiers are forced to pilot mechs in a brutal, racially-segregated war of survival.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -5157,6 +5482,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>An orphaned girl is taken in by a family cursed to turn into Zodiac animals when hugged by the opposite sex.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -5227,6 +5557,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>A law student suffering from amnesia must navigate his new college life, romance, and his forgotten past.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -5297,6 +5632,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>A young girl wanders into a magical world of spirits and must work in a bathhouse to free her parents.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -5367,6 +5707,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>A group of death-row convicts are sent to a beautiful but deadly island to find the elixir of life.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -5437,6 +5782,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>A single mother struggles to raise two half-wolf children while hiding their secret from society.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -5507,6 +5857,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>A college student survives a deadly attack but becomes a half-ghoul, forced to consume human flesh to survive.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -5577,6 +5932,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>An incredibly powerful hero who can defeat any opponent with a single punch struggles to find a challenge.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -5647,6 +6007,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>The weakest hunter of mankind gains a mysterious system that allows him to level up endlessly.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -5717,6 +6082,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>A young boy sets out on a perilous journey to become a Hunter and find his legendary father.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -5787,6 +6157,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Two brothers use forbidden alchemy in an attempt to resurrect their mother, leading to a quest for the Philosopher's Stone.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -5857,6 +6232,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>An elf mage reflects on life, time, and relationships after completing a legendary decade-long quest.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -5927,6 +6307,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>A short but incredibly athletic high schooler aims to revitalize his school's once-great volleyball team.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -5997,6 +6382,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>A clumsy boy is constantly protected by his cool, incredibly capable, and adorable girlfriend.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -6067,6 +6457,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>An otaku recruits an ordinary classmate to be the heroine of his ultimate dating sim game.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -6137,6 +6532,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>A high schooler must date powerful "Spirits" and make them fall in love to prevent catastrophic spatial quakes.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -6207,6 +6607,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>An incredibly powerful teenager tries to live a normal high school life while hiding his god-like abilities.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -6277,6 +6682,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>A soothing, slice-of-life journey through delicious cooking and heartwarming human connections.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -6347,6 +6757,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Two best friends navigate the messy boundaries between platonic friendship and romantic feelings.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -6417,6 +6832,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>A calm and composed girl reveals a surprisingly wild and lovable side whenever she drinks.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -6487,6 +6907,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>A high school girl uses her drama club acting skills to play different "harem" archetypes for her crush.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -6557,6 +6982,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>A former "chuunibyou" tries to live a normal high school life but is dragged into the delusions of a quirky classmate.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -6627,6 +7057,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>A quiet student befriends the slightly less popular, but far more interesting, girl in his class.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -6697,6 +7132,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Students at an elite girls' school secretly clash in highly competitive arcade fighting games.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -6767,6 +7207,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>The heirs of two rival gang factions must pretend to be dating to prevent an all-out war.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -6837,6 +7282,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>A complex story of music, romance, and time-traveling regrets in a small Japanese town.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -6907,6 +7357,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>Three childhood friends build a plane to reach a mysterious tower in an alternate-history divided Japan.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -6977,6 +7432,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>An unemployed 27-year-old is given a pill that makes him look 17 so he can redo his final year of high school.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -7047,6 +7507,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>A young girl who loves reading discovers her true passion for writing while falling for an aspiring violin maker.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -7117,6 +7582,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>A high school girl discovers she can literally leap backwards through time and uses it for trivial things.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -7187,6 +7657,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>A country boy joins a group of assassins to overthrow a deeply corrupt and ruthless empire.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -7257,6 +7732,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>A boy who hears voices is recruited into an intergalactic space police force.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -7327,6 +7807,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>The dark, visually stunning prequel to the Monogatari series exploring a boy's fateful encounter with a vampire.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -7397,6 +7882,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>A half-youmu boy meets a spirit warrior girl who uses her cursed blood as a weapon.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -7467,6 +7957,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>Four high school girls revive the light music club, drinking tea and slowly becoming a real band.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -7537,6 +8032,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>A sweet, misunderstood girl who looks like Sadako from The Ring slowly makes friends and finds love.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -7607,6 +8107,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>A magical, heartwarming mystery about finding letters from a secret friend at a new school.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -7677,6 +8182,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>A young woman from Tokyo accidentally becomes the "Queen" of a struggling rural town's tourism board.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -7747,6 +8257,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>A diligent student must tutor two genius girls in their weakest subjects to secure a scholarship.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -7817,6 +8332,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>Teens in an afterlife purgatory form a rebellion against God while trying to resolve their lingering regrets.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -7887,6 +8407,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>An immortal orb takes the form of things it encounters, learning about humanity through love and loss.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -7957,6 +8482,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>A poignant short film about fleeting summer memories and unbroken promises.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -8025,6 +8555,11 @@
       <c r="Q107" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>A devoted boy suddenly gives up on his crush, causing her to realize she actually misses his attention.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "fix: restore missing anime metadata and refine description panel layout"
This reverts commit 3dacca0299ba27218e1491d7b06599d5ba468366.
</commit_message>
<xml_diff>
--- a/assets/data/anime.xlsx
+++ b/assets/data/anime.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R107"/>
+  <dimension ref="A1:Q107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -502,11 +502,6 @@
           <t>Fav</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -580,11 +575,6 @@
       <c r="Q2" t="inlineStr">
         <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Two teenagers share a profound, magical connection upon discovering they are swapping bodies.</t>
         </is>
       </c>
     </row>
@@ -662,11 +652,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>A young girl teams up with a mysterious young man to close magical doors causing disasters across Japan.</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -742,11 +727,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>An aloof boy discovers his popular classmate is secretly suffering from a fatal pancreatic illness.</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -822,11 +802,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>A runaway high school boy in Tokyo meets a girl who has the power to manipulate the weather.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -902,11 +877,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>A student aspiring to be a shoemaker and a mysterious older woman find solace in each other on rainy mornings.</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -982,11 +952,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>Two seemingly very different high schoolers discover each other's hidden sides and form a close bond.</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1062,11 +1027,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>A kind-hearted boy becomes a demon slayer to avenge his family and cure his demon-turned sister.</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1142,11 +1102,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>A piano prodigy who lost his ability to hear the piano meets a free-spirited violinist who brings color back to his life.</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1222,11 +1177,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>Two teenagers investigate a mysterious tunnel that can grant wishes, but at a heavy cost of time.</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1302,11 +1252,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>A surfer and a firefighter fall in love, but tragedy strikes, leading to supernatural encounters.</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1382,11 +1327,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>A poignant tale of two childhood friends drifting apart over time and distance.</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1462,11 +1402,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>A high schooler helps girls suffering from "Puberty Syndrome," starting with a forgotten teen actress.</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1542,11 +1477,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>A doll-artisan enthusiast helps his popular classmate create cosplay outfits, blossoming into a sweet romance.</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1622,11 +1552,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>A young girl befriends a forest spirit who will disappear forever if touched by a human.</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1702,11 +1627,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>Two eccentric high schoolers get entangled in insane battles involving ghosts and aliens.</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1782,11 +1702,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>A beautifully animated reimagining of the classic Japanese folktale of the Bamboo Cutter.</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1862,11 +1777,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>A sci-fi romance exploring parallel universes and the choices that define true love.</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1942,11 +1852,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>The companion piece to "To Every You", showing the alternate universe path of love and sacrifice.</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2022,11 +1927,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>A street kid survives in a technology-obsessed city of the future by becoming a mercenary outlaw.</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2102,11 +2002,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>Set in the League of Legends universe, two sisters fight on rival sides of a war between two cities.</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2182,11 +2077,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>A former bully seeks redemption by trying to befriend the deaf girl he tormented in elementary school.</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2257,11 +2147,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>A heartbreaking story of two siblings struggling to survive in Japan during the final months of WWII.</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2332,11 +2217,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>A girl who lost her voice magically after traumatizing her family learns to express herself through music.</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2407,11 +2287,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>Humanity fights for survival against terrifying giant humanoids known as Titans.</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2482,11 +2357,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>Childhood friends from a sea village must attend school on the surface, causing friction and romance.</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2557,11 +2427,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>An energy-conserving high schooler joins the classic literature club and solves everyday mysteries.</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2632,11 +2497,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>In a post-apocalyptic future, children pilot giant mechs to defend humanity against monstrous threats.</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2707,11 +2567,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>A young man is transported to a fantasy world with the ability to rewind time upon his death.</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2782,11 +2637,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>A group of friends explore the nature of fireworks while a boy uses a mysterious orb to alter time.</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2857,11 +2707,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>A high schooler travels back in time to help his past self correct a mistake and save his love.</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2932,11 +2777,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>Three troubled teens seek out an urban legend known as the Summer Ghost to find answers about life and death.</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -3007,11 +2847,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>A beautiful, emotional one-shot about the complicated rivalry and friendship of two aspiring manga artists.</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -3082,11 +2917,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>A young viking warrior seeks revenge against the man who killed his father in a deeply philosophical historical epic.</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -3157,11 +2987,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>A brilliant high school student discovers a supernatural notebook that kills anyone whose name is written in it.</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3232,11 +3057,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>A delinquent student finds meaning in life by helping a sweet, chronically ill girl revive the school drama club.</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -3307,11 +3127,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>Two students suffering from insomnia find comfort in each other and the school's abandoned observatory.</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -3382,11 +3197,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>A sharp-witted apothecary girl solves medical mysteries and political intrigue within the Emperor's inner palace.</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -3457,11 +3267,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>A high schooler consumes a cursed talisman and gets drawn into a dangerous world of Curses and Sorcerers.</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -3532,11 +3337,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>Childhood friends reconnect years later to help the spirit of their deceased friend pass on.</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -3607,11 +3407,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>Two awkward coworkers fake an engagement to avoid being transferred to a branch office in Siberia.</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3682,11 +3477,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>A sweet sports romance about a badminton player and a basketball star living under the same roof.</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3757,11 +3547,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>An apathetic high school boy is slowly won over by his perfect, angelic neighbor who starts cooking for him.</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -3832,11 +3617,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>A socially awkward boy with dark fantasies slowly falls in love with the quirky, popular girl in his class.</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3907,11 +3687,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>Two mismatched students are paired up for a bizarre "marriage practical" assignment in school.</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3982,11 +3757,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t>Two brilliant student council leaders try to trick each other into confessing their love first.</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -4057,11 +3827,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>Two mismatched high schoolers team up to help each other confess to their respective crushes.</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -4132,11 +3897,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R48" t="inlineStr">
-        <is>
-          <t>A man travels back in time to his childhood to solve a string of kidnappings and save his classmate.</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -4207,11 +3967,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>Students in an ultra-competitive, cutthroat high school must use deception and strategy to rise to the top.</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -4282,11 +4037,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R50" t="inlineStr">
-        <is>
-          <t>A spy, an assassin, and a telepathic child pretend to be a normal family for a high-stakes mission.</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -4357,11 +4107,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>A beautiful half-Russian girl mutters sweet things in Russian, unaware that her crush perfectly understands her.</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -4432,11 +4177,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>A heartwarming romance between a student at a boys' delinquent school and a girl from an elite academy.</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -4507,11 +4247,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R53" t="inlineStr">
-        <is>
-          <t>A young woman cursed with an old body gets swept up in the magical world of a wizard named Howl.</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -4582,11 +4317,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R54" t="inlineStr">
-        <is>
-          <t>A young man merges with his pet chainsaw devil and joins a government agency to hunt other devils.</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -4657,11 +4387,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R55" t="inlineStr">
-        <is>
-          <t>A boy constantly finds himself comforting the girls who lose the "love triangles" in his school.</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -4732,11 +4457,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R56" t="inlineStr">
-        <is>
-          <t>A marine biology student becomes the caretaker for a stubborn, wheelchair-bound artist with big dreams.</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -4807,11 +4527,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R57" t="inlineStr">
-        <is>
-          <t>A happy alien tries to bring joy to a deeply traumatized human girl, leading to a dark tragedy.</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -4882,11 +4597,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R58" t="inlineStr">
-        <is>
-          <t>A touching drama about connection and finding light in a dark world.</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -4957,11 +4667,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R59" t="inlineStr">
-        <is>
-          <t>A comedic misunderstanding between two friends leads to unexpected romance.</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -5032,11 +4737,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R60" t="inlineStr">
-        <is>
-          <t>An emotional drama focused on terminal illness, love, and living life to the fullest.</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -5107,11 +4807,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R61" t="inlineStr">
-        <is>
-          <t>Childhood friends must navigate their shifting feelings and break the cycle of a complicated game.</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -5182,11 +4877,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R62" t="inlineStr">
-        <is>
-          <t>A secret organization of highly trained schoolgirls works in the shadows to maintain peace in Japan.</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -5257,11 +4947,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R63" t="inlineStr">
-        <is>
-          <t>A fierce delinquent joins a high school famous for brawling to fight for the town's safety.</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -5332,11 +5017,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R64" t="inlineStr">
-        <is>
-          <t>A soul is given a second chance at life inhabiting the body of a suicidal middle schooler.</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -5407,11 +5087,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R65" t="inlineStr">
-        <is>
-          <t>Child soldiers are forced to pilot mechs in a brutal, racially-segregated war of survival.</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -5482,11 +5157,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R66" t="inlineStr">
-        <is>
-          <t>An orphaned girl is taken in by a family cursed to turn into Zodiac animals when hugged by the opposite sex.</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -5557,11 +5227,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R67" t="inlineStr">
-        <is>
-          <t>A law student suffering from amnesia must navigate his new college life, romance, and his forgotten past.</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -5632,11 +5297,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R68" t="inlineStr">
-        <is>
-          <t>A young girl wanders into a magical world of spirits and must work in a bathhouse to free her parents.</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -5707,11 +5367,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R69" t="inlineStr">
-        <is>
-          <t>A group of death-row convicts are sent to a beautiful but deadly island to find the elixir of life.</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -5782,11 +5437,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R70" t="inlineStr">
-        <is>
-          <t>A single mother struggles to raise two half-wolf children while hiding their secret from society.</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -5857,11 +5507,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R71" t="inlineStr">
-        <is>
-          <t>A college student survives a deadly attack but becomes a half-ghoul, forced to consume human flesh to survive.</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -5932,11 +5577,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R72" t="inlineStr">
-        <is>
-          <t>An incredibly powerful hero who can defeat any opponent with a single punch struggles to find a challenge.</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -6007,11 +5647,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R73" t="inlineStr">
-        <is>
-          <t>The weakest hunter of mankind gains a mysterious system that allows him to level up endlessly.</t>
-        </is>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -6082,11 +5717,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R74" t="inlineStr">
-        <is>
-          <t>A young boy sets out on a perilous journey to become a Hunter and find his legendary father.</t>
-        </is>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -6157,11 +5787,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R75" t="inlineStr">
-        <is>
-          <t>Two brothers use forbidden alchemy in an attempt to resurrect their mother, leading to a quest for the Philosopher's Stone.</t>
-        </is>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -6232,11 +5857,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R76" t="inlineStr">
-        <is>
-          <t>An elf mage reflects on life, time, and relationships after completing a legendary decade-long quest.</t>
-        </is>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -6307,11 +5927,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R77" t="inlineStr">
-        <is>
-          <t>A short but incredibly athletic high schooler aims to revitalize his school's once-great volleyball team.</t>
-        </is>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -6382,11 +5997,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R78" t="inlineStr">
-        <is>
-          <t>A clumsy boy is constantly protected by his cool, incredibly capable, and adorable girlfriend.</t>
-        </is>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -6457,11 +6067,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R79" t="inlineStr">
-        <is>
-          <t>An otaku recruits an ordinary classmate to be the heroine of his ultimate dating sim game.</t>
-        </is>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -6532,11 +6137,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R80" t="inlineStr">
-        <is>
-          <t>A high schooler must date powerful "Spirits" and make them fall in love to prevent catastrophic spatial quakes.</t>
-        </is>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -6607,11 +6207,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R81" t="inlineStr">
-        <is>
-          <t>An incredibly powerful teenager tries to live a normal high school life while hiding his god-like abilities.</t>
-        </is>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -6682,11 +6277,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R82" t="inlineStr">
-        <is>
-          <t>A soothing, slice-of-life journey through delicious cooking and heartwarming human connections.</t>
-        </is>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -6757,11 +6347,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R83" t="inlineStr">
-        <is>
-          <t>Two best friends navigate the messy boundaries between platonic friendship and romantic feelings.</t>
-        </is>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -6832,11 +6417,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R84" t="inlineStr">
-        <is>
-          <t>A calm and composed girl reveals a surprisingly wild and lovable side whenever she drinks.</t>
-        </is>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -6907,11 +6487,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R85" t="inlineStr">
-        <is>
-          <t>A high school girl uses her drama club acting skills to play different "harem" archetypes for her crush.</t>
-        </is>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -6982,11 +6557,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R86" t="inlineStr">
-        <is>
-          <t>A former "chuunibyou" tries to live a normal high school life but is dragged into the delusions of a quirky classmate.</t>
-        </is>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -7057,11 +6627,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R87" t="inlineStr">
-        <is>
-          <t>A quiet student befriends the slightly less popular, but far more interesting, girl in his class.</t>
-        </is>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -7132,11 +6697,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R88" t="inlineStr">
-        <is>
-          <t>Students at an elite girls' school secretly clash in highly competitive arcade fighting games.</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -7207,11 +6767,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R89" t="inlineStr">
-        <is>
-          <t>The heirs of two rival gang factions must pretend to be dating to prevent an all-out war.</t>
-        </is>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -7282,11 +6837,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R90" t="inlineStr">
-        <is>
-          <t>A complex story of music, romance, and time-traveling regrets in a small Japanese town.</t>
-        </is>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -7357,11 +6907,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R91" t="inlineStr">
-        <is>
-          <t>Three childhood friends build a plane to reach a mysterious tower in an alternate-history divided Japan.</t>
-        </is>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -7432,11 +6977,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R92" t="inlineStr">
-        <is>
-          <t>An unemployed 27-year-old is given a pill that makes him look 17 so he can redo his final year of high school.</t>
-        </is>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -7507,11 +7047,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R93" t="inlineStr">
-        <is>
-          <t>A young girl who loves reading discovers her true passion for writing while falling for an aspiring violin maker.</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -7582,11 +7117,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R94" t="inlineStr">
-        <is>
-          <t>A high school girl discovers she can literally leap backwards through time and uses it for trivial things.</t>
-        </is>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -7657,11 +7187,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R95" t="inlineStr">
-        <is>
-          <t>A country boy joins a group of assassins to overthrow a deeply corrupt and ruthless empire.</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -7732,11 +7257,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R96" t="inlineStr">
-        <is>
-          <t>A boy who hears voices is recruited into an intergalactic space police force.</t>
-        </is>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -7807,11 +7327,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R97" t="inlineStr">
-        <is>
-          <t>The dark, visually stunning prequel to the Monogatari series exploring a boy's fateful encounter with a vampire.</t>
-        </is>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -7882,11 +7397,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R98" t="inlineStr">
-        <is>
-          <t>A half-youmu boy meets a spirit warrior girl who uses her cursed blood as a weapon.</t>
-        </is>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -7957,11 +7467,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R99" t="inlineStr">
-        <is>
-          <t>Four high school girls revive the light music club, drinking tea and slowly becoming a real band.</t>
-        </is>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -8032,11 +7537,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R100" t="inlineStr">
-        <is>
-          <t>A sweet, misunderstood girl who looks like Sadako from The Ring slowly makes friends and finds love.</t>
-        </is>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -8107,11 +7607,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R101" t="inlineStr">
-        <is>
-          <t>A magical, heartwarming mystery about finding letters from a secret friend at a new school.</t>
-        </is>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -8182,11 +7677,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R102" t="inlineStr">
-        <is>
-          <t>A young woman from Tokyo accidentally becomes the "Queen" of a struggling rural town's tourism board.</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -8257,11 +7747,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R103" t="inlineStr">
-        <is>
-          <t>A diligent student must tutor two genius girls in their weakest subjects to secure a scholarship.</t>
-        </is>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -8332,11 +7817,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R104" t="inlineStr">
-        <is>
-          <t>Teens in an afterlife purgatory form a rebellion against God while trying to resolve their lingering regrets.</t>
-        </is>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -8407,11 +7887,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R105" t="inlineStr">
-        <is>
-          <t>An immortal orb takes the form of things it encounters, learning about humanity through love and loss.</t>
-        </is>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -8482,11 +7957,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R106" t="inlineStr">
-        <is>
-          <t>A poignant short film about fleeting summer memories and unbroken promises.</t>
-        </is>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -8555,11 +8025,6 @@
       <c r="Q107" t="inlineStr">
         <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="R107" t="inlineStr">
-        <is>
-          <t>A devoted boy suddenly gives up on his crush, causing her to realize she actually misses his attention.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: implement description panel as absolute sibling to prevent squishing
</commit_message>
<xml_diff>
--- a/assets/data/anime.xlsx
+++ b/assets/data/anime.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q107"/>
+  <dimension ref="A1:R107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -502,6 +502,11 @@
           <t>Fav</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -575,6 +580,11 @@
       <c r="Q2" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Two teenagers share a profound, magical connection upon discovering they are swapping bodies.</t>
         </is>
       </c>
     </row>
@@ -652,6 +662,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>A young girl teams up with a mysterious young man to close magical doors causing disasters across Japan.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -727,6 +742,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>An aloof boy discovers his popular classmate is secretly suffering from a fatal pancreatic illness.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -802,6 +822,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>A runaway high school boy in Tokyo meets a girl who has the power to manipulate the weather.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -877,6 +902,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>A student aspiring to be a shoemaker and a mysterious older woman find solace in each other on rainy mornings.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -952,6 +982,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Two seemingly very different high schoolers discover each other's hidden sides and form a close bond.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1027,6 +1062,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>A kind-hearted boy becomes a demon slayer to avenge his family and cure his demon-turned sister.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1102,6 +1142,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>A piano prodigy who lost his ability to hear the piano meets a free-spirited violinist who brings color back to his life.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1177,6 +1222,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Two teenagers investigate a mysterious tunnel that can grant wishes, but at a heavy cost of time.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1252,6 +1302,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>A surfer and a firefighter fall in love, but tragedy strikes, leading to supernatural encounters.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1327,6 +1382,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>A poignant tale of two childhood friends drifting apart over time and distance.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1402,6 +1462,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>A high schooler helps girls suffering from "Puberty Syndrome," starting with a forgotten teen actress.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1477,6 +1542,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>A doll-artisan enthusiast helps his popular classmate create cosplay outfits, blossoming into a sweet romance.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1552,6 +1622,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>A young girl befriends a forest spirit who will disappear forever if touched by a human.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1627,6 +1702,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Two eccentric high schoolers get entangled in insane battles involving ghosts and aliens.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1702,6 +1782,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>A beautifully animated reimagining of the classic Japanese folktale of the Bamboo Cutter.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1777,6 +1862,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>A sci-fi romance exploring parallel universes and the choices that define true love.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1852,6 +1942,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>The companion piece to "To Every You", showing the alternate universe path of love and sacrifice.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1927,6 +2022,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>A street kid survives in a technology-obsessed city of the future by becoming a mercenary outlaw.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2002,6 +2102,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Set in the League of Legends universe, two sisters fight on rival sides of a war between two cities.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2077,6 +2182,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>A former bully seeks redemption by trying to befriend the deaf girl he tormented in elementary school.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2147,6 +2257,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>A heartbreaking story of two siblings struggling to survive in Japan during the final months of WWII.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2217,6 +2332,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>A girl who lost her voice magically after traumatizing her family learns to express herself through music.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2287,6 +2407,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Humanity fights for survival against terrifying giant humanoids known as Titans.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2357,6 +2482,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Childhood friends from a sea village must attend school on the surface, causing friction and romance.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2427,6 +2557,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>An energy-conserving high schooler joins the classic literature club and solves everyday mysteries.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2497,6 +2632,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>In a post-apocalyptic future, children pilot giant mechs to defend humanity against monstrous threats.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2567,6 +2707,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>A young man is transported to a fantasy world with the ability to rewind time upon his death.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2637,6 +2782,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>A group of friends explore the nature of fireworks while a boy uses a mysterious orb to alter time.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2707,6 +2857,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>A high schooler travels back in time to help his past self correct a mistake and save his love.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2777,6 +2932,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Three troubled teens seek out an urban legend known as the Summer Ghost to find answers about life and death.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2847,6 +3007,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>A beautiful, emotional one-shot about the complicated rivalry and friendship of two aspiring manga artists.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2917,6 +3082,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>A young viking warrior seeks revenge against the man who killed his father in a deeply philosophical historical epic.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2987,6 +3157,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>A brilliant high school student discovers a supernatural notebook that kills anyone whose name is written in it.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3057,6 +3232,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>A delinquent student finds meaning in life by helping a sweet, chronically ill girl revive the school drama club.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -3127,6 +3307,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Two students suffering from insomnia find comfort in each other and the school's abandoned observatory.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -3197,6 +3382,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>A sharp-witted apothecary girl solves medical mysteries and political intrigue within the Emperor's inner palace.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -3267,6 +3457,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>A high schooler consumes a cursed talisman and gets drawn into a dangerous world of Curses and Sorcerers.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -3337,6 +3532,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Childhood friends reconnect years later to help the spirit of their deceased friend pass on.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -3407,6 +3607,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Two awkward coworkers fake an engagement to avoid being transferred to a branch office in Siberia.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3477,6 +3682,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>A sweet sports romance about a badminton player and a basketball star living under the same roof.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3547,6 +3757,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>An apathetic high school boy is slowly won over by his perfect, angelic neighbor who starts cooking for him.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -3617,6 +3832,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>A socially awkward boy with dark fantasies slowly falls in love with the quirky, popular girl in his class.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3687,6 +3907,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Two mismatched students are paired up for a bizarre "marriage practical" assignment in school.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3757,6 +3982,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Two brilliant student council leaders try to trick each other into confessing their love first.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -3827,6 +4057,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Two mismatched high schoolers team up to help each other confess to their respective crushes.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3897,6 +4132,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>A man travels back in time to his childhood to solve a string of kidnappings and save his classmate.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3967,6 +4207,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Students in an ultra-competitive, cutthroat high school must use deception and strategy to rise to the top.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -4037,6 +4282,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>A spy, an assassin, and a telepathic child pretend to be a normal family for a high-stakes mission.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -4107,6 +4357,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>A beautiful half-Russian girl mutters sweet things in Russian, unaware that her crush perfectly understands her.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -4177,6 +4432,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>A heartwarming romance between a student at a boys' delinquent school and a girl from an elite academy.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -4247,6 +4507,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>A young woman cursed with an old body gets swept up in the magical world of a wizard named Howl.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -4317,6 +4582,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>A young man merges with his pet chainsaw devil and joins a government agency to hunt other devils.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -4387,6 +4657,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>A boy constantly finds himself comforting the girls who lose the "love triangles" in his school.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -4457,6 +4732,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>A marine biology student becomes the caretaker for a stubborn, wheelchair-bound artist with big dreams.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -4527,6 +4807,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>A happy alien tries to bring joy to a deeply traumatized human girl, leading to a dark tragedy.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -4597,6 +4882,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>A touching drama about connection and finding light in a dark world.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -4667,6 +4957,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>A comedic misunderstanding between two friends leads to unexpected romance.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -4737,6 +5032,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>An emotional drama focused on terminal illness, love, and living life to the fullest.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -4807,6 +5107,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Childhood friends must navigate their shifting feelings and break the cycle of a complicated game.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -4877,6 +5182,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>A secret organization of highly trained schoolgirls works in the shadows to maintain peace in Japan.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -4947,6 +5257,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>A fierce delinquent joins a high school famous for brawling to fight for the town's safety.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -5017,6 +5332,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>A soul is given a second chance at life inhabiting the body of a suicidal middle schooler.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -5087,6 +5407,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Child soldiers are forced to pilot mechs in a brutal, racially-segregated war of survival.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -5157,6 +5482,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>An orphaned girl is taken in by a family cursed to turn into Zodiac animals when hugged by the opposite sex.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -5227,6 +5557,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>A law student suffering from amnesia must navigate his new college life, romance, and his forgotten past.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -5297,6 +5632,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>A young girl wanders into a magical world of spirits and must work in a bathhouse to free her parents.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -5367,6 +5707,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>A group of death-row convicts are sent to a beautiful but deadly island to find the elixir of life.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -5437,6 +5782,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>A single mother struggles to raise two half-wolf children while hiding their secret from society.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -5507,6 +5857,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>A college student survives a deadly attack but becomes a half-ghoul, forced to consume human flesh to survive.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -5577,6 +5932,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>An incredibly powerful hero who can defeat any opponent with a single punch struggles to find a challenge.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -5647,6 +6007,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>The weakest hunter of mankind gains a mysterious system that allows him to level up endlessly.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -5717,6 +6082,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>A young boy sets out on a perilous journey to become a Hunter and find his legendary father.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -5787,6 +6157,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Two brothers use forbidden alchemy in an attempt to resurrect their mother, leading to a quest for the Philosopher's Stone.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -5857,6 +6232,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>An elf mage reflects on life, time, and relationships after completing a legendary decade-long quest.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -5927,6 +6307,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>A short but incredibly athletic high schooler aims to revitalize his school's once-great volleyball team.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -5997,6 +6382,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>A clumsy boy is constantly protected by his cool, incredibly capable, and adorable girlfriend.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -6067,6 +6457,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>An otaku recruits an ordinary classmate to be the heroine of his ultimate dating sim game.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -6137,6 +6532,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>A high schooler must date powerful "Spirits" and make them fall in love to prevent catastrophic spatial quakes.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -6207,6 +6607,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>An incredibly powerful teenager tries to live a normal high school life while hiding his god-like abilities.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -6277,6 +6682,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>A soothing, slice-of-life journey through delicious cooking and heartwarming human connections.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -6347,6 +6757,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Two best friends navigate the messy boundaries between platonic friendship and romantic feelings.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -6417,6 +6832,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>A calm and composed girl reveals a surprisingly wild and lovable side whenever she drinks.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -6487,6 +6907,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>A high school girl uses her drama club acting skills to play different "harem" archetypes for her crush.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -6557,6 +6982,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>A former "chuunibyou" tries to live a normal high school life but is dragged into the delusions of a quirky classmate.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -6627,6 +7057,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>A quiet student befriends the slightly less popular, but far more interesting, girl in his class.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -6697,6 +7132,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Students at an elite girls' school secretly clash in highly competitive arcade fighting games.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -6767,6 +7207,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>The heirs of two rival gang factions must pretend to be dating to prevent an all-out war.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -6837,6 +7282,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>A complex story of music, romance, and time-traveling regrets in a small Japanese town.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -6907,6 +7357,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>Three childhood friends build a plane to reach a mysterious tower in an alternate-history divided Japan.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -6977,6 +7432,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>An unemployed 27-year-old is given a pill that makes him look 17 so he can redo his final year of high school.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -7047,6 +7507,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>A young girl who loves reading discovers her true passion for writing while falling for an aspiring violin maker.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -7117,6 +7582,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>A high school girl discovers she can literally leap backwards through time and uses it for trivial things.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -7187,6 +7657,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>A country boy joins a group of assassins to overthrow a deeply corrupt and ruthless empire.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -7257,6 +7732,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>A boy who hears voices is recruited into an intergalactic space police force.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -7327,6 +7807,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>The dark, visually stunning prequel to the Monogatari series exploring a boy's fateful encounter with a vampire.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -7397,6 +7882,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>A half-youmu boy meets a spirit warrior girl who uses her cursed blood as a weapon.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -7467,6 +7957,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>Four high school girls revive the light music club, drinking tea and slowly becoming a real band.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -7537,6 +8032,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>A sweet, misunderstood girl who looks like Sadako from The Ring slowly makes friends and finds love.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -7607,6 +8107,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>A magical, heartwarming mystery about finding letters from a secret friend at a new school.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -7677,6 +8182,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>A young woman from Tokyo accidentally becomes the "Queen" of a struggling rural town's tourism board.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -7747,6 +8257,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>A diligent student must tutor two genius girls in their weakest subjects to secure a scholarship.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -7817,6 +8332,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>Teens in an afterlife purgatory form a rebellion against God while trying to resolve their lingering regrets.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -7887,6 +8407,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>An immortal orb takes the form of things it encounters, learning about humanity through love and loss.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -7957,6 +8482,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>A poignant short film about fleeting summer memories and unbroken promises.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -8025,6 +8555,11 @@
       <c r="Q107" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>A devoted boy suddenly gives up on his crush, causing her to realize she actually misses his attention.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(guide): update RDNDOBGS full franchise titles, years & 2 seasons breakdown
</commit_message>
<xml_diff>
--- a/assets/data/anime.xlsx
+++ b/assets/data/anime.xlsx
@@ -1410,7 +1410,7 @@
         </is>
       </c>
       <c r="H13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
         <v>13</v>
@@ -9024,1369 +9024,1369 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Rascal Does Not Dream of Bunny Girl Senpai</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Rascal Does Not Dream of Bunny Girl Senpai</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>TV Series</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Essential Canon</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>13 Episodes (2018)</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Covers Light Novel Vol 1–5: High School Arc (Mai, Tomoe, Rio, Nodoka, and Kaede arcs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Rascal Does Not Dream of Bunny Girl Senpai</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Rascal Does Not Dream of a Dreaming Girl</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Movie</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Essential Canon</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>89 Mins (2019)</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Covers Light Novel Vol 6–7. Direct continuation and emotional climax of Shoko Makinohara arc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Rascal Does Not Dream of Bunny Girl Senpai</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Rascal Does Not Dream of a Sister Venturing Out</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Movie</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Essential Canon</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>73 Mins (2023)</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Covers Light Novel Vol 8. Focuses on Kaede's recovery and high school entrance exam.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Rascal Does Not Dream of Bunny Girl Senpai</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Rascal Does Not Dream of a Knapsack Kid</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Movie</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Essential Canon</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>75 Mins (2023)</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Covers Light Novel Vol 9. Concludes the High School Arc with Mai &amp; young Shoko, leading to graduation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Rascal Does Not Dream of Bunny Girl Senpai</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Rascal Does Not Dream of Santa Claus</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>TV Series</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Essential Canon</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>13 Episodes (2025)</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Covers Light Novel Vol 10–12. Beginning of the University Arc (Touko Kirishima &amp; Miniskirt Santa).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Rascal Does Not Dream of Bunny Girl Senpai</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Rascal Does Not Dream of a Dear Friend</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Movie</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Upcoming Release</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Upcoming 2026</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Covers Light Novel Vol 13. Continuation of the University Arc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Demon Slayer</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Season 1: Tanjiro Kamado Arc</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>26 Episodes</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Beginning of Tanjiro's journey, Final Selection &amp; Mount Natagumo battle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Demon Slayer</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Mugen Train (Movie)</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Movie</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>117 Mins</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Direct canon continuation covering Rengoku &amp; Enmu. Choose Movie OR S2 TV Arc Part 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Demon Slayer</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>2b</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Mugen Train Arc (TV Version)</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Alternative</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>7 Episodes</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>TV cut of the movie. Ep 1 is an exclusive Rengoku backstory; Eps 2–7 match movie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Demon Slayer</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Season 2: Entertainment District Arc</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>11 Episodes</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Sound Hashira Tengen Uzui &amp; battle against Upper Rank 6 Daki and Gyutaro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Demon Slayer</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Season 3: Swordsmith Village Arc</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>11 Episodes</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Mist Hashira Muichiro &amp; Love Hashira Mitsuri in the hidden village.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Demon Slayer</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Season 4: Hashira Training Arc</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>8 Episodes</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Intensive Hashira training arc leading straight into the finale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Demon Slayer</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Infinity Castle Arc (Movie Trilogy)</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Movie</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Upcoming</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>3 Movies</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>The grand theatrical trilogy finale covering the final battle with Muzan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Chainsaw Man</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Season 1 (TV)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>TV Season</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>Essential</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>12 Episodes</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Covers Introduction up through the Katana Man Arc (Manga Ch. 1–38).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Chainsaw Man</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>1b</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Compilation Arc Parts 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Recap</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>2 Parts</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Recap of Season 1 with zero new story content. Safe to skip completely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Chainsaw Man</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Reze Arc (Movie)</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Movie</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Upcoming</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Canon continuation covering the Bomb Girl (Reze) Arc (Manga Ch. 39–52).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Attack on Titan</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Season 1 (TV)</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>25 Episodes</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Fall of Shiganshina, Battle of Trost, and Female Titan arc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Attack on Titan</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>1b</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Ilse's Notebook (OVA)</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>OVA</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>1 Episode</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Canon backstory revealing talking Titans, best watched right after Season 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Attack on Titan</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Season 2 (TV)</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>12 Episodes</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Clash of the Titans arc &amp; Beast Titan debut.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Attack on Titan</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>2b</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>No Regrets (OVA Parts 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>OVA</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>2 Episodes</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Levi Ackerman's canon underground backstory and Scout recruitment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Attack on Titan</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Season 3 Parts 1 &amp; 2 (TV)</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>22 Episodes</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Uprising Arc and the Return to Shiganshina / Basement reveal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Attack on Titan</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>The Final Season Parts 1 &amp; 2</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>28 Episodes</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Marley Arc &amp; War for Paradis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Attack on Titan</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>The Final Chapters (Specials 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>2 Specials (145 mins)</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>The Rumbling &amp; epic series conclusion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Jujutsu Kaisen</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Jujutsu Kaisen 0 (Movie)</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Movie</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>105 Mins</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Canon prequel film focusing on Yuta Okkotsu and Suguru Geto. Watch before S1 or between S1 and S2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Jujutsu Kaisen</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Season 1 (TV)</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>24 Episodes</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Yuji Itadori, Sukuna's fingers, and Kyoto Goodwill Event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Jujutsu Kaisen</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Season 2: Hidden Inventory &amp; Shibuya Incident</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>23 Episodes</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Gojo &amp; Geto's past (Eps 1–5), followed by the Shibuya Incident arc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Jujutsu Kaisen</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>The Culling Game Arc</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Upcoming</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Announced sequel following the catastrophic aftermath of Shibuya.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Kaguya-sama: Love Is War</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Season 1 (TV)</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>12 Episodes</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Introduction to the Student Council psychological warfare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Kaguya-sama: Love Is War</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Season 2 (TV)</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>12 Episodes</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Student council re-election and sports festival arc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Kaguya-sama: Love Is War</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>2b</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Kaguya-sama OVA</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>OVA</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>1 Episode (3 segments)</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Fanservice and comedy chapters; skip if only following romance progression.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Kaguya-sama: Love Is War</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Season 3: Ultra Romantic (TV)</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>13 Episodes</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Covers Light Novel Vol 1–5 (Mai, Tomoe, Rio, Nodoka, and Kaede arcs).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Rascal Does Not Dream of Bunny Girl Senpai</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>The cultural festival and dual confession climax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Kaguya-sama: Love Is War</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>The First Kiss That Never Ends</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Movie</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>96 Mins / 4 Eps</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Direct canon continuation exploring Kaguya and Miyuki's relationship post-festival.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Re:Zero</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Season 1 (TV / Director's Cut)</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Essential</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>25 Episodes</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Subaru's arrival in Lugunica and Return by Death introduction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Re:Zero</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>1b</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Memory Snow (OVA)</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>OVA</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>68 Mins</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Cozy canon slice-of-life side story set between Episode 11 and 12 of Season 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Re:Zero</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>1c</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>The Frozen Bond (OVA)</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>OVA</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>76 Mins</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Emilia and Puck's canon prequel backstory before meeting Subaru.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Re:Zero</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Dreaming Girl (Movie)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Movie</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Season 2 Parts 1 &amp; 2 (TV)</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
         <is>
           <t>Essential</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>89 Mins</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Direct continuation covering Vol 6–7. Emotional climax of Shoko Makinohara arc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Rascal Does Not Dream of Bunny Girl Senpai</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>25 Episodes</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>The Sanctuary arc and the Witches of Sin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>Re:Zero</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Sister Venturing Out (Movie)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Movie</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Season 3: Attack Arc &amp; Counterattack Arc</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>TV Season</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
         <is>
           <t>Essential</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>73 Mins</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Covers Vol 8. Focuses on Kaede's recovery and high school entrance exam.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Rascal Does Not Dream of Bunny Girl Senpai</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Knapsack Kid (Movie)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Movie</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>75 Mins</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Covers Vol 9. Concludes the High School Arc with Mai &amp; young Shoko.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Rascal Does Not Dream of Bunny Girl Senpai</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Season 2: University Arc (TV)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Upcoming</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Adapts the University Arc starting with Santa Claus (Vol 10+).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Rascal Does Not Dream of Bunny Girl Senpai</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Dear Friend (Movie)</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Movie</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Upcoming</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Future theatrical movie covering later University arc volumes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Demon Slayer</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Season 1: Tanjiro Kamado Arc</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>26 Episodes</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Beginning of Tanjiro's journey, Final Selection &amp; Mount Natagumo battle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Demon Slayer</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Mugen Train (Movie)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Movie</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Recommended</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>117 Mins</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Direct canon continuation covering Rengoku &amp; Enmu. Choose Movie OR S2 TV Arc Part 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Demon Slayer</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2b</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Mugen Train Arc (TV Version)</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Alternative</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>7 Episodes</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>TV cut of the movie. Ep 1 is an exclusive Rengoku backstory; Eps 2–7 match movie.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Demon Slayer</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Season 2: Entertainment District Arc</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>11 Episodes</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Sound Hashira Tengen Uzui &amp; battle against Upper Rank 6 Daki and Gyutaro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Demon Slayer</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Season 3: Swordsmith Village Arc</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>11 Episodes</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Mist Hashira Muichiro &amp; Love Hashira Mitsuri in the hidden village.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Demon Slayer</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Season 4: Hashira Training Arc</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>8 Episodes</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Intensive Hashira training arc leading straight into the finale.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Demon Slayer</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Infinity Castle Arc (Movie Trilogy)</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Movie</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Upcoming</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>3 Movies</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>The grand theatrical trilogy finale covering the final battle with Muzan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Chainsaw Man</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Season 1 (TV)</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>12 Episodes</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Covers Introduction up through the Katana Man Arc (Manga Ch. 1–38).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Chainsaw Man</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>1b</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Compilation Arc Parts 1 &amp; 2</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Recap</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Skip</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>2 Parts</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Recap of Season 1 with zero new story content. Safe to skip completely.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Chainsaw Man</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Reze Arc (Movie)</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Movie</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Upcoming</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Canon continuation covering the Bomb Girl (Reze) Arc (Manga Ch. 39–52).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Attack on Titan</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Season 1 (TV)</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>25 Episodes</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Fall of Shiganshina, Battle of Trost, and Female Titan arc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Attack on Titan</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>1b</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Ilse's Notebook (OVA)</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>OVA</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Recommended</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>1 Episode</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Canon backstory revealing talking Titans, best watched right after Season 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Attack on Titan</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Season 2 (TV)</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>12 Episodes</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Clash of the Titans arc &amp; Beast Titan debut.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Attack on Titan</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>2b</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>No Regrets (OVA Parts 1 &amp; 2)</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>OVA</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Recommended</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>2 Episodes</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Levi Ackerman's canon underground backstory and Scout recruitment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Attack on Titan</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Season 3 Parts 1 &amp; 2 (TV)</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>22 Episodes</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Uprising Arc and the Return to Shiganshina / Basement reveal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Attack on Titan</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>The Final Season Parts 1 &amp; 2</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>28 Episodes</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Marley Arc &amp; War for Paradis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Attack on Titan</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>The Final Chapters (Specials 1 &amp; 2)</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Special</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>2 Specials (145 mins)</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>The Rumbling &amp; epic series conclusion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Jujutsu Kaisen</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Jujutsu Kaisen 0 (Movie)</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Movie</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Recommended</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>105 Mins</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Canon prequel film focusing on Yuta Okkotsu and Suguru Geto. Watch before S1 or between S1 and S2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Jujutsu Kaisen</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Season 1 (TV)</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>24 Episodes</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Yuji Itadori, Sukuna's fingers, and Kyoto Goodwill Event.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Jujutsu Kaisen</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Season 2: Hidden Inventory &amp; Shibuya Incident</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>23 Episodes</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Gojo &amp; Geto's past (Eps 1–5), followed by the Shibuya Incident arc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Jujutsu Kaisen</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>The Culling Game Arc</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Upcoming</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Announced sequel following the catastrophic aftermath of Shibuya.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Kaguya-sama: Love Is War</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Season 1 (TV)</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>12 Episodes</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Introduction to the Student Council psychological warfare.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Kaguya-sama: Love Is War</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Season 2 (TV)</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>12 Episodes</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Student council re-election and sports festival arc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Kaguya-sama: Love Is War</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>2b</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Kaguya-sama OVA</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>OVA</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>1 Episode (3 segments)</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Fanservice and comedy chapters; skip if only following romance progression.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Kaguya-sama: Love Is War</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Season 3: Ultra Romantic (TV)</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>13 Episodes</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>The cultural festival and dual confession climax.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Kaguya-sama: Love Is War</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>The First Kiss That Never Ends</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Movie</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>96 Mins / 4 Eps</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Direct canon continuation exploring Kaguya and Miyuki's relationship post-festival.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Re:Zero</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Season 1 (TV / Director's Cut)</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>25 Episodes</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Subaru's arrival in Lugunica and Return by Death introduction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Re:Zero</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>1b</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Memory Snow (OVA)</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>OVA</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>68 Mins</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Cozy canon slice-of-life side story set between Episode 11 and 12 of Season 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Re:Zero</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>1c</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>The Frozen Bond (OVA)</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>OVA</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Recommended</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>76 Mins</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Emilia and Puck's canon prequel backstory before meeting Subaru.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Re:Zero</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Season 2 Parts 1 &amp; 2 (TV)</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>25 Episodes</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>The Sanctuary arc and the Witches of Sin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Re:Zero</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Season 3: Attack Arc &amp; Counterattack Arc</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>TV Season</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Essential</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="7" t="inlineStr">
         <is>
           <t>16 Episodes</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G38" s="7" t="inlineStr">
         <is>
           <t>Water City Priestella and Sin Archbishops invasion.</t>
         </is>

</xml_diff>